<commit_message>
Show usage of the new function to list cached object keys
</commit_message>
<xml_diff>
--- a/basics/passing_objects.xlsx
+++ b/basics/passing_objects.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25629"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github\xlslim-code-samples\basics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1434933C-25DC-4A73-B8B8-23AB05772C28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B925710D-C628-44BE-93E1-5F3758675ECC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{257F9B7E-B69A-46EF-8C88-E8306DB661FD}"/>
+    <workbookView xWindow="5666" yWindow="531" windowWidth="24883" windowHeight="15275" xr2:uid="{257F9B7E-B69A-46EF-8C88-E8306DB661FD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -31,6 +31,7 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -60,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
   <si>
     <t>Workbook location</t>
   </si>
@@ -125,6 +126,12 @@
   </si>
   <si>
     <t>Here we create Person objects by directly constructing Python classes, no factory function is required.</t>
+  </si>
+  <si>
+    <t>Cached Object Keys</t>
+  </si>
+  <si>
+    <t>The keys of all cached objects are returned by the =ListCachedKeys() function</t>
   </si>
 </sst>
 </file>
@@ -345,9 +352,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -385,7 +392,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -491,7 +498,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -633,7 +640,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -641,7 +648,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{774E7E1C-D275-4DD4-9028-FA14541EA3B8}">
-  <dimension ref="A1:M26"/>
+  <dimension ref="A1:M35"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="30.3046875" customWidth="1"/>
@@ -679,7 +686,7 @@
       </c>
       <c r="B3" s="3" t="str" cm="1">
         <f t="array" ref="B3">_xll.RegisterPyModule(B2)</f>
-        <v>Initialised the Python environment at C:\Users\russe\anaconda3\envs\py38. Registered D:\github\xlslim-code-samples\basics\passing_objects.py</v>
+        <v>Registered D:\github\xlslim-code-samples\basics\passing_objects.py</v>
       </c>
       <c r="G3" s="1"/>
     </row>
@@ -757,38 +764,38 @@
       </c>
       <c r="B9" s="3" t="str" cm="1">
         <f t="array" ref="B9">_xll.create_person(B6,B7,B8)</f>
-        <v>[passing_objects.xlsx]Sheet1$B$9@1</v>
+        <v>[passing_objects.xlsx]Sheet1$B$9/72277DA4@2</v>
       </c>
       <c r="C9" s="3" t="str" cm="1">
         <f t="array" ref="C9">_xll.create_person(C6,C7,C8)</f>
-        <v>[passing_objects.xlsx]Sheet1$C$9@1</v>
+        <v>[passing_objects.xlsx]Sheet1$C$9/6AF728A7@2</v>
       </c>
       <c r="D9" s="3" t="str" cm="1">
         <f t="array" ref="D9">_xll.create_person(D6,D7,D8)</f>
-        <v>[passing_objects.xlsx]Sheet1$D$9@1</v>
+        <v>[passing_objects.xlsx]Sheet1$D$9/9F2C3B05@2</v>
       </c>
       <c r="E9" s="3" t="str" cm="1">
         <f t="array" ref="E9">_xll.create_person(E6,E7,E8)</f>
-        <v>[passing_objects.xlsx]Sheet1$E$9@1</v>
+        <v>[passing_objects.xlsx]Sheet1$E$9/626FAF0F@2</v>
       </c>
       <c r="G9" s="5" t="s">
         <v>15</v>
       </c>
       <c r="H9" s="3" t="str" cm="1">
         <f t="array" ref="H9">_xll.Person(B6,B7,B8)</f>
-        <v>[passing_objects.xlsx]Sheet1$H$9@1</v>
+        <v>[passing_objects.xlsx]Sheet1$H$9/97F43B12@2</v>
       </c>
       <c r="I9" s="3" t="str" cm="1">
         <f t="array" ref="I9">_xll.Person(C6,C7,C8)</f>
-        <v>[passing_objects.xlsx]Sheet1$I$9@1</v>
+        <v>[passing_objects.xlsx]Sheet1$I$9/90D4E5FA@2</v>
       </c>
       <c r="J9" s="3" t="str" cm="1">
         <f t="array" ref="J9">_xll.Person(D6,D7,D8)</f>
-        <v>[passing_objects.xlsx]Sheet1$J$9@1</v>
+        <v>[passing_objects.xlsx]Sheet1$J$9/C500786B@3</v>
       </c>
       <c r="K9" s="3" t="str" cm="1">
         <f t="array" ref="K9">_xll.Person(E6,E7,E8)</f>
-        <v>[passing_objects.xlsx]Sheet1$K$9@1</v>
+        <v>[passing_objects.xlsx]Sheet1$K$9/88356C84@2</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.4">
@@ -994,10 +1001,67 @@
       <c r="G26" s="12"/>
       <c r="H26" s="13"/>
     </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A28" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B28" s="3" t="str" cm="1">
+        <f t="array" ref="B28:B35">_xll.ListCachedKeys()</f>
+        <v>[passing_objects.xlsx]Sheet1$K$9/88356C84</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="E28" s="8"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="B29" s="3" t="str">
+        <v>[passing_objects.xlsx]Sheet1$I$9/90D4E5FA</v>
+      </c>
+      <c r="D29" s="10"/>
+      <c r="E29" s="10"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="B30" s="3" t="str">
+        <v>[passing_objects.xlsx]Sheet1$H$9/97F43B12</v>
+      </c>
+      <c r="D30" s="10"/>
+      <c r="E30" s="10"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="B31" s="3" t="str">
+        <v>[passing_objects.xlsx]Sheet1$E$9/626FAF0F</v>
+      </c>
+      <c r="D31" s="10"/>
+      <c r="E31" s="10"/>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="B32" s="3" t="str">
+        <v>[passing_objects.xlsx]Sheet1$B$9/72277DA4</v>
+      </c>
+      <c r="D32" s="10"/>
+      <c r="E32" s="10"/>
+    </row>
+    <row r="33" spans="2:2" x14ac:dyDescent="0.4">
+      <c r="B33" s="3" t="str">
+        <v>[passing_objects.xlsx]Sheet1$C$9/6AF728A7</v>
+      </c>
+    </row>
+    <row r="34" spans="2:2" x14ac:dyDescent="0.4">
+      <c r="B34" s="3" t="str">
+        <v>[passing_objects.xlsx]Sheet1$D$9/9F2C3B05</v>
+      </c>
+    </row>
+    <row r="35" spans="2:2" x14ac:dyDescent="0.4">
+      <c r="B35" s="3" t="str">
+        <v>[passing_objects.xlsx]Sheet1$J$9/C500786B</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A13:H26"/>
     <mergeCell ref="G6:K7"/>
+    <mergeCell ref="D28:E32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1005,9 +1069,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1143,26 +1210,15 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5B898F4E-8707-4CA2-9F8B-513D2A3B8BD6}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FE1A4A2-BF99-4D94-B73F-D9211460B53D}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="a95c0ba0-d2e6-4b25-b7d5-a719ecc5544a"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1186,9 +1242,17 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FE1A4A2-BF99-4D94-B73F-D9211460B53D}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5B898F4E-8707-4CA2-9F8B-513D2A3B8BD6}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a95c0ba0-d2e6-4b25-b7d5-a719ecc5544a"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>